<commit_message>
Update cluster_vergleich Excel outputs (5 existing customers)
Refreshed with new NK exact-path loading and extended CUSTOMERS dict.

https://claude.ai/code/session_01QY1f1VNnd5RWsUcy3L3Squ
</commit_message>
<xml_diff>
--- a/output/cluster_vergleich/423650_HERMA_GmbH_cluster.xlsx
+++ b/output/cluster_vergleich/423650_HERMA_GmbH_cluster.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="HERMA GmbH" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="NK_Konditionen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23557,4 +23558,1281 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Schlüssel</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Aktiv</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Aktive 
+Sendung 
+in Import- 
+/Export-
+Land</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Prüfung ERKA</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>wird geprüft 
+von</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>betrifft
+Abrechnung</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>betrifft
+Erfassung
+(manuell)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>betrifft
+EDI</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>betrifft
+Operative/
+Abfertigung</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Filler2</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>DFÜ 
+ja / Nein</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Bemerkungen AX-Team</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Umsatz 2024 P1-P9</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>PSS</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>PSS Umsatz 2024-2025</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Name, Straße, LKZ, PLZ Ort</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Check Sendung 2024-2025</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Column2
+SSS Satzart → Transportart:
+•1 – National
+•2 – Import
+•3 – Export
+•0 – Nicht 
+relevant</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Land</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Bemerkung / Hinweis für AX</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Benutzergruppe
+•0 - Alle Benutzer     
+•5 - Abrechnung debitorisch 
+•6 - Abrechnung kreditorisch
+•1 / 2 / 3 / 4 / 8 – Nicht relevant</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Prüfungshinweis
+grün -&gt; in AX hinterlegt
+pink-&gt; in AX zu hinterlegen
+rot -&gt; in AX nicht relevant
+orange -&gt; in AX Routing prüfen/umsetzen
+blau -&gt; EDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>485112I</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>3 - wird benötigt in der Abrechnung</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>EDI</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>1364579.499999998</v>
+      </c>
+      <c r="N2" t="n">
+        <v>48511</v>
+      </c>
+      <c r="O2" t="n">
+        <v>48511</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>HERMA GMBH / LIEF.NR. 103988,  HEINRICH-HERMANN-STRASSE 14,  D  70794  FILDERSTADT BONLANDEN</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>485112I</t>
+        </is>
+      </c>
+      <c r="R2" t="n">
+        <v>2</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>doppelt</t>
+        </is>
+      </c>
+      <c r="U2" t="n">
+        <v>5</v>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>&gt; LADEMETER ABRECHNEN ! | &gt; BEI MASCHINENTEILE = 18002 VERWENDEN !</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>485113GB</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>EDI</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>1364579.499999998</v>
+      </c>
+      <c r="N3" t="n">
+        <v>48511</v>
+      </c>
+      <c r="O3" t="n">
+        <v>48511</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>HERMA GMBH / LIEF.NR. 103988,  HEINRICH-HERMANN-STRASSE 14,  D  70794  FILDERSTADT BONLANDEN</t>
+        </is>
+      </c>
+      <c r="R3" t="n">
+        <v>3</v>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>keine aktive SDG in 2024</t>
+        </is>
+      </c>
+      <c r="U3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>&gt; COUNTY LABELS LTD. --&gt; "COU01" |   BITTE DIESE KD.-NR. VERWENDEN !! | &gt; KEIN DIREKTZUSTELLUNGSKENNZEICHEN SETZTEN !!! | &gt; CCL WELLINGBOROUGH IMMER EINBUCHEN: |   Amelia: uk.transport@avery.com |   Corrie: cviljoen@avery.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>485113I</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0 - unklar, kann aus Abrechnungssicht nicht eingeordnet werden</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>EDI</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>1364579.499999998</v>
+      </c>
+      <c r="N4" t="n">
+        <v>48511</v>
+      </c>
+      <c r="O4" t="n">
+        <v>48511</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>HERMA GMBH / LIEF.NR. 103988,  HEINRICH-HERMANN-STRASSE 14,  D  70794  FILDERSTADT BONLANDEN</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>485113I</t>
+        </is>
+      </c>
+      <c r="R4" t="n">
+        <v>3</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Hinweis für Operative (aus 2012?)</t>
+        </is>
+      </c>
+      <c r="U4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>&gt; SDG. FÜR PILOT, CORNATE D'ADDA -&gt; FAHRER MUSS |   PALETTEN AN BORDKANTE BEREITSTELLEN -&gt; KEINE |   KOFFERVERLADUNGEN !!!!! (05.12.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>485113F</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2 - wird benötigt in der Abrechnung - betrifft aber auch Erfassung</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>EDI</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>1364579.499999998</v>
+      </c>
+      <c r="N5" t="n">
+        <v>48511</v>
+      </c>
+      <c r="O5" t="n">
+        <v>48511</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>HERMA GMBH / LIEF.NR. 103988,  HEINRICH-HERMANN-STRASSE 14,  D  70794  FILDERSTADT BONLANDEN</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>485113F</t>
+        </is>
+      </c>
+      <c r="R5" t="n">
+        <v>3</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>betrifft EDI</t>
+        </is>
+      </c>
+      <c r="U5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | &gt; EMPFÄNGER : TECHMAY, F-12100 MILLAU |   = 1,5 FACHE AN BENÖTIGTEN LADEMETER ERFASSEN !!</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>210973</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>4 - betrifft Erfassung/ Abfertigung/ Operative</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>EDI</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>84607.77000000002</v>
+      </c>
+      <c r="N6" t="n">
+        <v>21097</v>
+      </c>
+      <c r="O6" t="n">
+        <v>21097</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>HERMA GMBH / LIEF.NR. 103988,  HEINRICH-HERMANN-STRASSE 14,  D  70794  FILDERSTADT</t>
+        </is>
+      </c>
+      <c r="R6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>AN RAMPE 24 DARF NUR NOCH MIT UNSEREM NV GELADEN | WERDEN. | BITTE KEINEN UNTERNEHMER HINSCHICKEN. | .</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>485113</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2 - wird benötigt in der Abrechnung - betrifft aber auch Erfassung</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>EDI</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>1364579.499999998</v>
+      </c>
+      <c r="N7" t="n">
+        <v>48511</v>
+      </c>
+      <c r="O7" t="n">
+        <v>48511</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>HERMA GMBH / LIEF.NR. 103988,  HEINRICH-HERMANN-STRASSE 14,  D  70794  FILDERSTADT BONLANDEN</t>
+        </is>
+      </c>
+      <c r="R7" t="n">
+        <v>3</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>doppelt</t>
+        </is>
+      </c>
+      <c r="U7" t="n">
+        <v>5</v>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>&gt; BEI KOMPLETTE BITTE 24000KG FRPFL. ERFASSEN !</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>485112I</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0 - unklar, kann aus Abrechnungssicht nicht eingeordnet werden</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>EDI</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>1364579.499999998</v>
+      </c>
+      <c r="N8" t="n">
+        <v>48511</v>
+      </c>
+      <c r="O8" t="n">
+        <v>48511</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>HERMA GMBH / LIEF.NR. 103988,  HEINRICH-HERMANN-STRASSE 14,  D  70794  FILDERSTADT BONLANDEN</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>485112I</t>
+        </is>
+      </c>
+      <c r="R8" t="n">
+        <v>2</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>betrifft EDI</t>
+        </is>
+      </c>
+      <c r="U8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>&gt; BITTE IMMER LM ERFASSEN !! | &gt; 48511 = HAFTMATERIAL/ETTIKETTEN |   18002 = MASCHINENTEILE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>408103</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>4 - betrifft Erfassung/ Abfertigung/ Operative</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>EDI</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>19228.5</v>
+      </c>
+      <c r="N9" t="n">
+        <v>40810</v>
+      </c>
+      <c r="O9" t="n">
+        <v>40810</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>HERMA GMBH / LIEF.NR. 103988,  HEINRICH-HERMANN-STRASSE 14,  D  70794  FILDERSTADT</t>
+        </is>
+      </c>
+      <c r="R9" t="n">
+        <v>3</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>AN RAMPE 24 DARF NUR NOCH MIT ERKA-NV GELADEN | WERDEN | BITTE KEINEN UNTERNEHMER HINSCHICKEN. | .</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>408103GB</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>EDI</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>19228.5</v>
+      </c>
+      <c r="N10" t="n">
+        <v>40810</v>
+      </c>
+      <c r="O10" t="n">
+        <v>40810</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>HERMA GMBH / LIEF.NR. 103988,  HEINRICH-HERMANN-STRASSE 14,  D  70794  FILDERSTADT</t>
+        </is>
+      </c>
+      <c r="R10" t="n">
+        <v>3</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>keine aktive SDG in 2024</t>
+        </is>
+      </c>
+      <c r="U10" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>COUNTY LABELS LTD. --&gt; "COU01" | BITTE DIESE KD.-NR. VERWENDEN !! | --&gt; KEIN DIREKTZUSTELLUNGSKENNZEICHEN SETZTEN !!! | LM SIND EIN PLFICHTFELD, DIES GILT ABER NUR FÜR | KUNDENSPERRIGKEIT -&gt; BEI PARTNER DÜRFT IHR GERNE | CBM EINGEBEN, VOR ALLEM BEI EINZELNEN KARTONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>408103I</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>3 - wird benötigt in der Abrechnung</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>EDI</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>19228.5</v>
+      </c>
+      <c r="N11" t="n">
+        <v>40810</v>
+      </c>
+      <c r="O11" t="n">
+        <v>40810</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>HERMA GMBH / LIEF.NR. 103988,  HEINRICH-HERMANN-STRASSE 14,  D  70794  FILDERSTADT</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>408103I</t>
+        </is>
+      </c>
+      <c r="R11" t="n">
+        <v>3</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>noch aktuell? Falls ja, bitte nähere Infos.</t>
+        </is>
+      </c>
+      <c r="U11" t="n">
+        <v>5</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>BITTE BEI KOMPLETTEN LKW'S AUFPASSEN UND GGF. | 20000 KG ALS FRACHTPFLICHTIGES GEWICHT ERFASSEN | DASS DIE OFFERTE DEN KOMPLETTPREIS RECHNET | *** | SENDUNGEN FÜR STAPLES CASTELETTO - HIER SIND | STANDZEITEN VOM PARTNER IN ORDNUNG - HERMA IST | INFORMIERT,DASS WIR ABRECHNEN-09/13 HR.GRANZA | AN HERMA (ORDNER RALI/LOTUS/HERMA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>485113</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>0 - unklar, kann aus Abrechnungssicht nicht eingeordnet werden</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>EDI</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>1364579.5</v>
+      </c>
+      <c r="N12" t="n">
+        <v>48511</v>
+      </c>
+      <c r="O12" t="n">
+        <v>48511</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>HERMA GMBH / LIEF.NR. 103988,  HEINRICH-HERMANN-STRASSE 14,  D  70794  FILDERSTADT BONLANDEN</t>
+        </is>
+      </c>
+      <c r="R12" t="n">
+        <v>3</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Hinweis für Operative offen
+Abrechnungshinweis erledigt</t>
+        </is>
+      </c>
+      <c r="U12" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>&gt; AN RAMPE 24 DARF NUR NOCH MIT UNSEREM NV GELADEN |   WERDEN. | &gt; BITTE KEINEN UNTERNEHMER HINSCHICKEN. | &gt; BEI KOMPLETTE BITTE 24000KG FRPFL. ERFASSEN !</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>180023</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>4 - betrifft Erfassung/ Abfertigung/ Operative</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>EDI</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>5534.629999999998</v>
+      </c>
+      <c r="N13" t="n">
+        <v>18002</v>
+      </c>
+      <c r="O13" t="n">
+        <v>18002</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>HERMA GMBH,  HEINRICH-HERMANN-STRASSE 14,  D  70794  FILDERSTADT</t>
+        </is>
+      </c>
+      <c r="R13" t="n">
+        <v>3</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>AN RAMPE 24 DARF NUR NOCH MIT UNSEREM NV GELADEN | WERDEN. | BITTE KEINEN UNTERNEHMER HINSCHICKEN. | .</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>180023F</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>4 - betrifft Erfassung/ Abfertigung/ Operative</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>EDI</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>5534.629999999998</v>
+      </c>
+      <c r="N14" t="n">
+        <v>18002</v>
+      </c>
+      <c r="O14" t="n">
+        <v>18002</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>HERMA GMBH,  HEINRICH-HERMANN-STRASSE 14,  D  70794  FILDERSTADT</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>180023F</t>
+        </is>
+      </c>
+      <c r="R14" t="n">
+        <v>3</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="U14" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>WENN FRANKATUR FCA BITTE MIT HERMA KLÄREN OB | HERMA,F 67930 BEINHEIM FZ IST - WENN JA DANN | FRANKATUR 89 ERFASSEN UND 15256 ALS ABW FZ ERFASSE | N</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>180023GB</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>EDI</t>
+        </is>
+      </c>
+      <c r="M15" t="n">
+        <v>5534.629999999998</v>
+      </c>
+      <c r="N15" t="n">
+        <v>18002</v>
+      </c>
+      <c r="O15" t="n">
+        <v>18002</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>HERMA GMBH,  HEINRICH-HERMANN-STRASSE 14,  D  70794  FILDERSTADT</t>
+        </is>
+      </c>
+      <c r="R15" t="n">
+        <v>3</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>keine aktive SDG in 2024</t>
+        </is>
+      </c>
+      <c r="U15" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>&gt; SENDUNGEN ZU HERMA HAVERHILL |   ENTWEDER FRANKATUR 89 ERFASSEN ODER |   HERMA HAVERHILL ALS ABW.FZ IN FELD 7 ERFASSEN &amp; |   FRANKATUR FREI HAUS (94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>210973I</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2 - wird benötigt in der Abrechnung - betrifft aber auch Erfassung</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>EDI</t>
+        </is>
+      </c>
+      <c r="M16" t="n">
+        <v>84607.77000000002</v>
+      </c>
+      <c r="N16" t="n">
+        <v>21097</v>
+      </c>
+      <c r="O16" t="n">
+        <v>21097</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>HERMA GMBH / LIEF.NR. 103988,  HEINRICH-HERMANN-STRASSE 14,  D  70794  FILDERSTADT</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>210973I</t>
+        </is>
+      </c>
+      <c r="R16" t="n">
+        <v>3</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Hinweis für Operative offen
+Abrechnungshinweis offen</t>
+        </is>
+      </c>
+      <c r="U16" t="n">
+        <v>6</v>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>SDG. F. AUTOMATION ADDR... IN MONZA SIND IMMER | UNFREI - WENN GRUBER UNSERE ABR. NICHT AKZEPTIERT | EINFACH WIEDER ZURÜCKBELASTEN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>408102GB</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>EDI</t>
+        </is>
+      </c>
+      <c r="M17" t="n">
+        <v>19228.5</v>
+      </c>
+      <c r="N17" t="n">
+        <v>40810</v>
+      </c>
+      <c r="O17" t="n">
+        <v>40810</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>HERMA GMBH / LIEF.NR. 103988,  HEINRICH-HERMANN-STRASSE 14,  D  70794  FILDERSTADT</t>
+        </is>
+      </c>
+      <c r="R17" t="n">
+        <v>2</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>keine aktive SDG in 2024</t>
+        </is>
+      </c>
+      <c r="U17" t="n">
+        <v>6</v>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>EXPORTPREISE | AUSFUHR EURO 65,00  // VERZOLLUNG EURO 15,00 | RÜCKWARE EURO 65,00 | ZOLLBESCHAU EURO 25,00 | LOGISTIK.SERVICE@HERMA.DE, NICOLE.THUERING@HERMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>180023I</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>4 - betrifft Erfassung/ Abfertigung/ Operative</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>EDI</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>5534.629999999998</v>
+      </c>
+      <c r="N18" t="n">
+        <v>18002</v>
+      </c>
+      <c r="O18" t="n">
+        <v>18002</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>HERMA GMBH,  HEINRICH-HERMANN-STRASSE 14,  D  70794  FILDERSTADT</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>180023I</t>
+        </is>
+      </c>
+      <c r="R18" t="n">
+        <v>3</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="U18" t="n">
+        <v>6</v>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>SDG. F. AUTOMATION ADDR... IN MONZA SIND IMMER | UNFREI - GRUBER BELASTET STÄNDIG UNSERE ABR. ZURÜC | K. KANN ZURÜCKBELASTET WERDEN OHNE ÜBERPRÜFUNG | DER ABTEILUNG</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>580022I</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="n">
+        <v>58002</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>HERMA GMBH,  PLOCHINGER STR. 48,  D  73779  DEIZISAU</t>
+        </is>
+      </c>
+      <c r="R19" t="n">
+        <v>2</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>keine aktive SDG in 2024</t>
+        </is>
+      </c>
+      <c r="U19" t="n">
+        <v>5</v>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>NEUE OFFERTE ANGELEGT AUS PLZ 42 30.08.17 | DARF KEINE AT-MAUT RECHNEN. | KANN WENN KORREKT GELÖSCHT WERDEN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>580023GB</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="n">
+        <v>58002</v>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>HERMA GMBH,  PLOCHINGER STR. 48,  D  73779  DEIZISAU</t>
+        </is>
+      </c>
+      <c r="R20" t="n">
+        <v>3</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>keine aktive SDG in 2024</t>
+        </is>
+      </c>
+      <c r="U20" t="n">
+        <v>0</v>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>SENDUNGEN SIND FAST IMMER UNFREI --&gt; | ALSO BITTE DIE LM VOR ALLEM IN DIE SSP EINGEBEN</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>